<commit_message>
Merge beard and moustache transplants into one treatment
Old beard/moustache URLs redirect to the combined page (refresh page on
GitHub Pages, 301 via _redirects on Cloudflare Pages).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HXTFKm4ap8ug2QKhDLkwhp
</commit_message>
<xml_diff>
--- a/elite-plus/_docs/Elite-Plus-Clinic-Data-Intake.xlsx
+++ b/elite-plus/_docs/Elite-Plus-Clinic-Data-Intake.xlsx
@@ -690,7 +690,7 @@
         </is>
       </c>
       <c r="B17" s="7">
-        <f>COUNTA('Treatments'!C6:F16)/(ROWS('Treatments'!C6:F16)*COLUMNS('Treatments'!C6:F16))</f>
+        <f>COUNTA('Treatments'!C6:F15)/(ROWS('Treatments'!C6:F15)*COLUMNS('Treatments'!C6:F15))</f>
         <v/>
       </c>
     </row>
@@ -701,7 +701,7 @@
         </is>
       </c>
       <c r="B18" s="7">
-        <f>COUNTA('Treatment content'!B6:G16)/(ROWS('Treatment content'!B6:G16)*COLUMNS('Treatment content'!B6:G16))</f>
+        <f>COUNTA('Treatment content'!B6:G15)/(ROWS('Treatment content'!B6:G15)*COLUMNS('Treatment content'!B6:G15))</f>
         <v/>
       </c>
     </row>
@@ -2931,7 +2931,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F19"/>
+  <dimension ref="A1:F18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -3044,7 +3044,7 @@
       </c>
       <c r="B7" s="10" t="inlineStr">
         <is>
-          <t>Beard Transplant</t>
+          <t>Beard &amp; Moustache Transplant</t>
         </is>
       </c>
       <c r="C7" s="12" t="n"/>
@@ -3076,7 +3076,7 @@
       </c>
       <c r="B9" s="10" t="inlineStr">
         <is>
-          <t>Moustache Transplant</t>
+          <t>Scar Hair Transplant</t>
         </is>
       </c>
       <c r="C9" s="12" t="n"/>
@@ -3092,7 +3092,7 @@
       </c>
       <c r="B10" s="10" t="inlineStr">
         <is>
-          <t>Scar Hair Transplant</t>
+          <t>Burn Scar Hair Transplant</t>
         </is>
       </c>
       <c r="C10" s="12" t="n"/>
@@ -3103,12 +3103,12 @@
     <row r="11">
       <c r="A11" s="10" t="inlineStr">
         <is>
-          <t>Hair Transplant</t>
+          <t>Hair Treatments</t>
         </is>
       </c>
       <c r="B11" s="10" t="inlineStr">
         <is>
-          <t>Burn Scar Hair Transplant</t>
+          <t>G-Cell Hair Therapy</t>
         </is>
       </c>
       <c r="C11" s="12" t="n"/>
@@ -3124,7 +3124,7 @@
       </c>
       <c r="B12" s="10" t="inlineStr">
         <is>
-          <t>G-Cell Hair Therapy</t>
+          <t>Stem Cell Hair Therapy</t>
         </is>
       </c>
       <c r="C12" s="12" t="n"/>
@@ -3140,7 +3140,7 @@
       </c>
       <c r="B13" s="10" t="inlineStr">
         <is>
-          <t>Stem Cell Hair Therapy</t>
+          <t>Regenera Activa (confirm name)</t>
         </is>
       </c>
       <c r="C13" s="12" t="n"/>
@@ -3156,7 +3156,7 @@
       </c>
       <c r="B14" s="10" t="inlineStr">
         <is>
-          <t>Regenera Activa (confirm name)</t>
+          <t>PRP (Plasma) Hair Treatment</t>
         </is>
       </c>
       <c r="C14" s="12" t="n"/>
@@ -3172,7 +3172,7 @@
       </c>
       <c r="B15" s="10" t="inlineStr">
         <is>
-          <t>PRP (Plasma) Hair Treatment</t>
+          <t>Hair Mesotherapy</t>
         </is>
       </c>
       <c r="C15" s="12" t="n"/>
@@ -3181,16 +3181,8 @@
       <c r="F15" s="12" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="10" t="inlineStr">
-        <is>
-          <t>Hair Treatments</t>
-        </is>
-      </c>
-      <c r="B16" s="10" t="inlineStr">
-        <is>
-          <t>Hair Mesotherapy</t>
-        </is>
-      </c>
+      <c r="A16" s="12" t="n"/>
+      <c r="B16" s="12" t="n"/>
       <c r="C16" s="12" t="n"/>
       <c r="D16" s="12" t="n"/>
       <c r="E16" s="12" t="n"/>
@@ -3211,14 +3203,6 @@
       <c r="D18" s="12" t="n"/>
       <c r="E18" s="12" t="n"/>
       <c r="F18" s="12" t="n"/>
-    </row>
-    <row r="19">
-      <c r="A19" s="12" t="n"/>
-      <c r="B19" s="12" t="n"/>
-      <c r="C19" s="12" t="n"/>
-      <c r="D19" s="12" t="n"/>
-      <c r="E19" s="12" t="n"/>
-      <c r="F19" s="12" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3232,7 +3216,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G16"/>
+  <dimension ref="A1:G15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -3352,7 +3336,7 @@
     <row r="7" ht="90" customHeight="1">
       <c r="A7" s="10" t="inlineStr">
         <is>
-          <t>Beard Transplant</t>
+          <t>Beard &amp; Moustache Transplant</t>
         </is>
       </c>
       <c r="B7" s="12" t="n"/>
@@ -3378,7 +3362,7 @@
     <row r="9" ht="90" customHeight="1">
       <c r="A9" s="10" t="inlineStr">
         <is>
-          <t>Moustache Transplant</t>
+          <t>Scar Hair Transplant</t>
         </is>
       </c>
       <c r="B9" s="12" t="n"/>
@@ -3391,7 +3375,7 @@
     <row r="10" ht="90" customHeight="1">
       <c r="A10" s="10" t="inlineStr">
         <is>
-          <t>Scar Hair Transplant</t>
+          <t>Burn Scar Hair Transplant</t>
         </is>
       </c>
       <c r="B10" s="12" t="n"/>
@@ -3404,7 +3388,7 @@
     <row r="11" ht="90" customHeight="1">
       <c r="A11" s="10" t="inlineStr">
         <is>
-          <t>Burn Scar Hair Transplant</t>
+          <t>G-Cell Hair Therapy</t>
         </is>
       </c>
       <c r="B11" s="12" t="n"/>
@@ -3417,7 +3401,7 @@
     <row r="12" ht="90" customHeight="1">
       <c r="A12" s="10" t="inlineStr">
         <is>
-          <t>G-Cell Hair Therapy</t>
+          <t>Stem Cell Hair Therapy</t>
         </is>
       </c>
       <c r="B12" s="12" t="n"/>
@@ -3430,7 +3414,7 @@
     <row r="13" ht="90" customHeight="1">
       <c r="A13" s="10" t="inlineStr">
         <is>
-          <t>Stem Cell Hair Therapy</t>
+          <t>Regenera Activa (confirm name)</t>
         </is>
       </c>
       <c r="B13" s="12" t="n"/>
@@ -3443,7 +3427,7 @@
     <row r="14" ht="90" customHeight="1">
       <c r="A14" s="10" t="inlineStr">
         <is>
-          <t>Regenera Activa (confirm name)</t>
+          <t>PRP (Plasma) Hair Treatment</t>
         </is>
       </c>
       <c r="B14" s="12" t="n"/>
@@ -3456,7 +3440,7 @@
     <row r="15" ht="90" customHeight="1">
       <c r="A15" s="10" t="inlineStr">
         <is>
-          <t>PRP (Plasma) Hair Treatment</t>
+          <t>Hair Mesotherapy</t>
         </is>
       </c>
       <c r="B15" s="12" t="n"/>
@@ -3465,19 +3449,6 @@
       <c r="E15" s="12" t="n"/>
       <c r="F15" s="12" t="n"/>
       <c r="G15" s="12" t="n"/>
-    </row>
-    <row r="16" ht="90" customHeight="1">
-      <c r="A16" s="10" t="inlineStr">
-        <is>
-          <t>Hair Mesotherapy</t>
-        </is>
-      </c>
-      <c r="B16" s="12" t="n"/>
-      <c r="C16" s="12" t="n"/>
-      <c r="D16" s="12" t="n"/>
-      <c r="E16" s="12" t="n"/>
-      <c r="F16" s="12" t="n"/>
-      <c r="G16" s="12" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Merge scar pages, transplant content, Turkey address, social buttons, remove reviews
- Scar & Burn Scar Hair Transplant is one page; old burn-scar URL redirects
- Researched intro, who it is for, steps, stay and FAQ for all transplants
- 7,000+ patients treated; Google ratings and review sections removed
- Türkiye clinic address as text (no map embed or map link); phone left empty
- Instagram/Facebook as brand-coloured buttons: floating stack with WhatsApp
  on desktop, beside WhatsApp in the header on phones and tablets; language
  list moves into the phone menu to make room

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HXTFKm4ap8ug2QKhDLkwhp
</commit_message>
<xml_diff>
--- a/elite-plus/_docs/Elite-Plus-Clinic-Data-Intake.xlsx
+++ b/elite-plus/_docs/Elite-Plus-Clinic-Data-Intake.xlsx
@@ -690,7 +690,7 @@
         </is>
       </c>
       <c r="B17" s="7">
-        <f>COUNTA('Treatments'!C6:F15)/(ROWS('Treatments'!C6:F15)*COLUMNS('Treatments'!C6:F15))</f>
+        <f>COUNTA('Treatments'!C6:F14)/(ROWS('Treatments'!C6:F14)*COLUMNS('Treatments'!C6:F14))</f>
         <v/>
       </c>
     </row>
@@ -701,7 +701,7 @@
         </is>
       </c>
       <c r="B18" s="7">
-        <f>COUNTA('Treatment content'!B6:G15)/(ROWS('Treatment content'!B6:G15)*COLUMNS('Treatment content'!B6:G15))</f>
+        <f>COUNTA('Treatment content'!B6:G14)/(ROWS('Treatment content'!B6:G14)*COLUMNS('Treatment content'!B6:G14))</f>
         <v/>
       </c>
     </row>
@@ -2931,7 +2931,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F18"/>
+  <dimension ref="A1:F17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -3076,7 +3076,7 @@
       </c>
       <c r="B9" s="10" t="inlineStr">
         <is>
-          <t>Scar Hair Transplant</t>
+          <t>Scar &amp; Burn Scar Hair Transplant</t>
         </is>
       </c>
       <c r="C9" s="12" t="n"/>
@@ -3087,12 +3087,12 @@
     <row r="10">
       <c r="A10" s="10" t="inlineStr">
         <is>
-          <t>Hair Transplant</t>
+          <t>Hair Treatments</t>
         </is>
       </c>
       <c r="B10" s="10" t="inlineStr">
         <is>
-          <t>Burn Scar Hair Transplant</t>
+          <t>G-Cell Hair Therapy</t>
         </is>
       </c>
       <c r="C10" s="12" t="n"/>
@@ -3108,7 +3108,7 @@
       </c>
       <c r="B11" s="10" t="inlineStr">
         <is>
-          <t>G-Cell Hair Therapy</t>
+          <t>Stem Cell Hair Therapy</t>
         </is>
       </c>
       <c r="C11" s="12" t="n"/>
@@ -3124,7 +3124,7 @@
       </c>
       <c r="B12" s="10" t="inlineStr">
         <is>
-          <t>Stem Cell Hair Therapy</t>
+          <t>Regenera Activa (confirm name)</t>
         </is>
       </c>
       <c r="C12" s="12" t="n"/>
@@ -3140,7 +3140,7 @@
       </c>
       <c r="B13" s="10" t="inlineStr">
         <is>
-          <t>Regenera Activa (confirm name)</t>
+          <t>PRP (Plasma) Hair Treatment</t>
         </is>
       </c>
       <c r="C13" s="12" t="n"/>
@@ -3156,7 +3156,7 @@
       </c>
       <c r="B14" s="10" t="inlineStr">
         <is>
-          <t>PRP (Plasma) Hair Treatment</t>
+          <t>Hair Mesotherapy</t>
         </is>
       </c>
       <c r="C14" s="12" t="n"/>
@@ -3165,16 +3165,8 @@
       <c r="F14" s="12" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="10" t="inlineStr">
-        <is>
-          <t>Hair Treatments</t>
-        </is>
-      </c>
-      <c r="B15" s="10" t="inlineStr">
-        <is>
-          <t>Hair Mesotherapy</t>
-        </is>
-      </c>
+      <c r="A15" s="12" t="n"/>
+      <c r="B15" s="12" t="n"/>
       <c r="C15" s="12" t="n"/>
       <c r="D15" s="12" t="n"/>
       <c r="E15" s="12" t="n"/>
@@ -3195,14 +3187,6 @@
       <c r="D17" s="12" t="n"/>
       <c r="E17" s="12" t="n"/>
       <c r="F17" s="12" t="n"/>
-    </row>
-    <row r="18">
-      <c r="A18" s="12" t="n"/>
-      <c r="B18" s="12" t="n"/>
-      <c r="C18" s="12" t="n"/>
-      <c r="D18" s="12" t="n"/>
-      <c r="E18" s="12" t="n"/>
-      <c r="F18" s="12" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3216,7 +3200,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G15"/>
+  <dimension ref="A1:G14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -3362,7 +3346,7 @@
     <row r="9" ht="90" customHeight="1">
       <c r="A9" s="10" t="inlineStr">
         <is>
-          <t>Scar Hair Transplant</t>
+          <t>Scar &amp; Burn Scar Hair Transplant</t>
         </is>
       </c>
       <c r="B9" s="12" t="n"/>
@@ -3375,7 +3359,7 @@
     <row r="10" ht="90" customHeight="1">
       <c r="A10" s="10" t="inlineStr">
         <is>
-          <t>Burn Scar Hair Transplant</t>
+          <t>G-Cell Hair Therapy</t>
         </is>
       </c>
       <c r="B10" s="12" t="n"/>
@@ -3388,7 +3372,7 @@
     <row r="11" ht="90" customHeight="1">
       <c r="A11" s="10" t="inlineStr">
         <is>
-          <t>G-Cell Hair Therapy</t>
+          <t>Stem Cell Hair Therapy</t>
         </is>
       </c>
       <c r="B11" s="12" t="n"/>
@@ -3401,7 +3385,7 @@
     <row r="12" ht="90" customHeight="1">
       <c r="A12" s="10" t="inlineStr">
         <is>
-          <t>Stem Cell Hair Therapy</t>
+          <t>Regenera Activa (confirm name)</t>
         </is>
       </c>
       <c r="B12" s="12" t="n"/>
@@ -3414,7 +3398,7 @@
     <row r="13" ht="90" customHeight="1">
       <c r="A13" s="10" t="inlineStr">
         <is>
-          <t>Regenera Activa (confirm name)</t>
+          <t>PRP (Plasma) Hair Treatment</t>
         </is>
       </c>
       <c r="B13" s="12" t="n"/>
@@ -3427,7 +3411,7 @@
     <row r="14" ht="90" customHeight="1">
       <c r="A14" s="10" t="inlineStr">
         <is>
-          <t>PRP (Plasma) Hair Treatment</t>
+          <t>Hair Mesotherapy</t>
         </is>
       </c>
       <c r="B14" s="12" t="n"/>
@@ -3436,19 +3420,6 @@
       <c r="E14" s="12" t="n"/>
       <c r="F14" s="12" t="n"/>
       <c r="G14" s="12" t="n"/>
-    </row>
-    <row r="15" ht="90" customHeight="1">
-      <c r="A15" s="10" t="inlineStr">
-        <is>
-          <t>Hair Mesotherapy</t>
-        </is>
-      </c>
-      <c r="B15" s="12" t="n"/>
-      <c r="C15" s="12" t="n"/>
-      <c r="D15" s="12" t="n"/>
-      <c r="E15" s="12" t="n"/>
-      <c r="F15" s="12" t="n"/>
-      <c r="G15" s="12" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Simplify site: clinic pages show details only; remove doctors, prices, licences, reviews
- Removed: eyebrow transplant page and results, first beard result, doctors
  section and pages, prices page and price panels, licence references,
  Facebook, home results and doctors sections, clinic filter and locations
  on results (old URLs redirect)
- Clinic pages: address, WhatsApp, phone, email, hours, video call, photos
- Results ordered as requested; 12-month follow-up; VIP transportation
- Telegram button next to Instagram/WhatsApp (link pending); smaller header
  icons on phones/tablets; flat design without drop shadows
- Phone/tablet: tighter spacing, 2-column categories on tablets, no
  duplicate WhatsApp button, header fits 320-1023px in all languages

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HXTFKm4ap8ug2QKhDLkwhp
</commit_message>
<xml_diff>
--- a/elite-plus/_docs/Elite-Plus-Clinic-Data-Intake.xlsx
+++ b/elite-plus/_docs/Elite-Plus-Clinic-Data-Intake.xlsx
@@ -690,7 +690,7 @@
         </is>
       </c>
       <c r="B17" s="7">
-        <f>COUNTA('Treatments'!C6:F14)/(ROWS('Treatments'!C6:F14)*COLUMNS('Treatments'!C6:F14))</f>
+        <f>COUNTA('Treatments'!C6:F13)/(ROWS('Treatments'!C6:F13)*COLUMNS('Treatments'!C6:F13))</f>
         <v/>
       </c>
     </row>
@@ -701,7 +701,7 @@
         </is>
       </c>
       <c r="B18" s="7">
-        <f>COUNTA('Treatment content'!B6:G14)/(ROWS('Treatment content'!B6:G14)*COLUMNS('Treatment content'!B6:G14))</f>
+        <f>COUNTA('Treatment content'!B6:G13)/(ROWS('Treatment content'!B6:G13)*COLUMNS('Treatment content'!B6:G13))</f>
         <v/>
       </c>
     </row>
@@ -2931,7 +2931,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F17"/>
+  <dimension ref="A1:F16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -3060,7 +3060,7 @@
       </c>
       <c r="B8" s="10" t="inlineStr">
         <is>
-          <t>Eyebrow Transplant</t>
+          <t>Scar &amp; Burn Scar Hair Transplant</t>
         </is>
       </c>
       <c r="C8" s="12" t="n"/>
@@ -3071,12 +3071,12 @@
     <row r="9">
       <c r="A9" s="10" t="inlineStr">
         <is>
-          <t>Hair Transplant</t>
+          <t>Hair Treatments</t>
         </is>
       </c>
       <c r="B9" s="10" t="inlineStr">
         <is>
-          <t>Scar &amp; Burn Scar Hair Transplant</t>
+          <t>G-Cell Hair Therapy</t>
         </is>
       </c>
       <c r="C9" s="12" t="n"/>
@@ -3092,7 +3092,7 @@
       </c>
       <c r="B10" s="10" t="inlineStr">
         <is>
-          <t>G-Cell Hair Therapy</t>
+          <t>Stem Cell Hair Therapy</t>
         </is>
       </c>
       <c r="C10" s="12" t="n"/>
@@ -3108,7 +3108,7 @@
       </c>
       <c r="B11" s="10" t="inlineStr">
         <is>
-          <t>Stem Cell Hair Therapy</t>
+          <t>Regenera Activa (confirm name)</t>
         </is>
       </c>
       <c r="C11" s="12" t="n"/>
@@ -3124,7 +3124,7 @@
       </c>
       <c r="B12" s="10" t="inlineStr">
         <is>
-          <t>Regenera Activa (confirm name)</t>
+          <t>PRP (Plasma) Hair Treatment</t>
         </is>
       </c>
       <c r="C12" s="12" t="n"/>
@@ -3140,7 +3140,7 @@
       </c>
       <c r="B13" s="10" t="inlineStr">
         <is>
-          <t>PRP (Plasma) Hair Treatment</t>
+          <t>Hair Mesotherapy</t>
         </is>
       </c>
       <c r="C13" s="12" t="n"/>
@@ -3149,16 +3149,8 @@
       <c r="F13" s="12" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="10" t="inlineStr">
-        <is>
-          <t>Hair Treatments</t>
-        </is>
-      </c>
-      <c r="B14" s="10" t="inlineStr">
-        <is>
-          <t>Hair Mesotherapy</t>
-        </is>
-      </c>
+      <c r="A14" s="12" t="n"/>
+      <c r="B14" s="12" t="n"/>
       <c r="C14" s="12" t="n"/>
       <c r="D14" s="12" t="n"/>
       <c r="E14" s="12" t="n"/>
@@ -3179,14 +3171,6 @@
       <c r="D16" s="12" t="n"/>
       <c r="E16" s="12" t="n"/>
       <c r="F16" s="12" t="n"/>
-    </row>
-    <row r="17">
-      <c r="A17" s="12" t="n"/>
-      <c r="B17" s="12" t="n"/>
-      <c r="C17" s="12" t="n"/>
-      <c r="D17" s="12" t="n"/>
-      <c r="E17" s="12" t="n"/>
-      <c r="F17" s="12" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3200,7 +3184,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G14"/>
+  <dimension ref="A1:G13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -3333,7 +3317,7 @@
     <row r="8" ht="90" customHeight="1">
       <c r="A8" s="10" t="inlineStr">
         <is>
-          <t>Eyebrow Transplant</t>
+          <t>Scar &amp; Burn Scar Hair Transplant</t>
         </is>
       </c>
       <c r="B8" s="12" t="n"/>
@@ -3346,7 +3330,7 @@
     <row r="9" ht="90" customHeight="1">
       <c r="A9" s="10" t="inlineStr">
         <is>
-          <t>Scar &amp; Burn Scar Hair Transplant</t>
+          <t>G-Cell Hair Therapy</t>
         </is>
       </c>
       <c r="B9" s="12" t="n"/>
@@ -3359,7 +3343,7 @@
     <row r="10" ht="90" customHeight="1">
       <c r="A10" s="10" t="inlineStr">
         <is>
-          <t>G-Cell Hair Therapy</t>
+          <t>Stem Cell Hair Therapy</t>
         </is>
       </c>
       <c r="B10" s="12" t="n"/>
@@ -3372,7 +3356,7 @@
     <row r="11" ht="90" customHeight="1">
       <c r="A11" s="10" t="inlineStr">
         <is>
-          <t>Stem Cell Hair Therapy</t>
+          <t>Regenera Activa (confirm name)</t>
         </is>
       </c>
       <c r="B11" s="12" t="n"/>
@@ -3385,7 +3369,7 @@
     <row r="12" ht="90" customHeight="1">
       <c r="A12" s="10" t="inlineStr">
         <is>
-          <t>Regenera Activa (confirm name)</t>
+          <t>PRP (Plasma) Hair Treatment</t>
         </is>
       </c>
       <c r="B12" s="12" t="n"/>
@@ -3398,7 +3382,7 @@
     <row r="13" ht="90" customHeight="1">
       <c r="A13" s="10" t="inlineStr">
         <is>
-          <t>PRP (Plasma) Hair Treatment</t>
+          <t>Hair Mesotherapy</t>
         </is>
       </c>
       <c r="B13" s="12" t="n"/>
@@ -3407,19 +3391,6 @@
       <c r="E13" s="12" t="n"/>
       <c r="F13" s="12" t="n"/>
       <c r="G13" s="12" t="n"/>
-    </row>
-    <row r="14" ht="90" customHeight="1">
-      <c r="A14" s="10" t="inlineStr">
-        <is>
-          <t>Hair Mesotherapy</t>
-        </is>
-      </c>
-      <c r="B14" s="12" t="n"/>
-      <c r="C14" s="12" t="n"/>
-      <c r="D14" s="12" t="n"/>
-      <c r="E14" s="12" t="n"/>
-      <c r="F14" s="12" t="n"/>
-      <c r="G14" s="12" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>